<commit_message>
Technical review corrections: align all documents on CNV and phasing language
- Corrected phasing description: BUB1B variants are unphased (GT:AD:DP:GQ:PL), PGT/PID present at nearby sites only
- Softened CNV language: regional mean depth is a coarse diploid-copy screen, not formal exclusion
- Removed inappropriate Jekel's citation for MHC artifacts
- Added FANCD2 as non-competing secondary candidate
- Aligned README, bitacora, report, methods Excel, and source scripts
- All 4 key corrections verified via grep (no residual problematic text)
</commit_message>
<xml_diff>
--- a/submission/JoseVelasco22_track1_methods.xlsx
+++ b/submission/JoseVelasco22_track1_methods.xlsx
@@ -469,6 +469,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
@@ -501,7 +502,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>We applied Exomiser v14.0.0 under three orthogonal configurations to verify robustness: (1) a targeted 22-gene panel of known MVA/microcephaly/SAC genes; (2) an expanded 51-gene panel adding DNA-repair and checkpoint genes (TP53, BRCA1/2, CHEK1/2, ATM, ATR); (3) a genome-wide run restricted to coding and splice-site variants via variantEffectFilter. BUB1B ranked first with identical combined score 0.9819 across all three configurations, demonstrating the finding does not depend on gene-set definition. We performed forensic validation of four potential limitations: (a) CNV exclusion via depth-of-coverage comparison (BUB1B 43.2x vs control 43.3x); (b) rejection of HLA-DRB1 as a false positive driven by MHC hyperpolymorphism; (c) phase inference by Mendelian functional parsimony (cis incompatible with recessive MVA phenotype); (d) promoter/UTR scan with no causal regulatory variants. Final submission is a compound heterozygous pair: chr15:40,209,701 T&gt;G (p.Leu737*, ClinVar PATHOGENIC, 2 stars) and chr15:40,220,612 T&gt;G (p.Asn1002Lys, VUS, AlphaMissense 0.923).</t>
+          <t>We applied Exomiser v14.0.0 under three orthogonal configurations to verify robustness: (1) a targeted 22-gene panel of known MVA/microcephaly/SAC genes; (2) an expanded 51-gene panel adding DNA-repair and checkpoint genes (TP53, BRCA1/2, CHEK1/2, ATM, ATR); (3) a genome-wide run restricted to coding and splice-site variants via variantEffectFilter. BUB1B ranked first with identical combined score 0.9819 across all three configurations, demonstrating the finding does not depend on gene-set definition. We performed forensic validation of four potential limitations: (a) coarse CNV screening via depth-of-coverage comparison (BUB1B 43.2x vs control 43.3x); (b) rejection of HLA-DRB1 as a false positive driven by MHC hyperpolymorphism; (c) phase inference by Mendelian functional parsimony (the two BUB1B variants are unphased in the VCF; cis incompatible with recessive MVA phenotype); (d) promoter/UTR scan with no causal regulatory variants. Final submission is a compound heterozygous pair: chr15:40,209,701 T&gt;G (p.Leu737*, ClinVar PATHOGENIC, 2 stars) and chr15:40,220,612 T&gt;G (p.Asn1002Lys, VUS, AlphaMissense 0.923).</t>
         </is>
       </c>
     </row>
@@ -537,7 +538,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Manual review consisted of evidence verification, not variant selection: (a) confirmed ClinVar ID 533901 for p.Leu737* with 2-star review status; (b) confirmed absence from ClinVar for p.Asn1002Lys (VUS); (c) inspected GATK PGT/PID tags in the VCF to confirm read-based phasing was unavailable (variants 10.9 kb apart exceed fragment size); (d) computed mean DP in BUB1B vs control region to exclude CNV; (e) identified HLA-DRB1 rank-2 signal as MHC hyperpolymorphism artifact.</t>
+          <t>Manual review consisted of evidence verification, not variant selection: (a) confirmed ClinVar ID 533901 for p.Leu737* with 2-star review status; (b) confirmed absence from ClinVar for p.Asn1002Lys (VUS); (c) inspected GATK PGT/PID tags in the VCF to confirm read-based phasing was unavailable (variants 10.9 kb apart exceed fragment size); (d) computed mean DP in BUB1B vs control region as a coarse CNV screen; small CNVs would require a dedicated SV/CNV caller; (e) identified HLA-DRB1 rank-2 signal as MHC hyperpolymorphism artifact.</t>
         </is>
       </c>
     </row>
@@ -622,7 +623,7 @@
       <c r="B17" s="3" t="inlineStr">
         <is>
           <t>We present an orthogonal-validation pipeline for rare-disease variant prioritization, applied to a single WGS proband with Mosaic Variegated Aneuploidy syndrome 1 (MVA1). The method is built on Exomiser v14.0.0 but goes beyond a single-run prioritization by executing three independent configurations — a 22-gene targeted panel, a 51-gene expanded panel, and a genome-wide coding+splice filter — and requiring convergence across all three before accepting a candidate. The primary finding, a BUB1B compound heterozygote (p.Leu737* + p.Asn1002Lys), achieved a combined score of 0.9819 in all three runs, demonstrating robustness to gene-set definition.
-Strengths: (1) orthogonal convergence eliminates panel-definition artifacts; (2) forensic validation of four common failure modes (CNV, MHC false positives, unphased compound hets, regulatory variants); (3) integration of ClinVar 2-star evidence as independent confirmation; (4) transparent declaration of discordant in-silico scores (AlphaMissense 0.923 vs REVEL 0.472); (5) low computational cost (~8 minutes, 6 GB heap, consumer laptop).
+Strengths: (1) orthogonal convergence eliminates panel-definition artifacts; (2) forensic validation of four common failure modes (coarse CNV assessment, MHC false positives, unphased compound hets, regulatory variants); (3) integration of ClinVar 2-star evidence as independent confirmation; (4) transparent declaration of discordant in-silico scores (AlphaMissense 0.923 vs REVEL 0.472); (5) low computational cost (~8 minutes, 6 GB heap, consumer laptop).
 Limitations: (1) phase is inferred by Mendelian functional parsimony rather than confirmed by read phasing or parental data; (2) p.Asn1002Lys remains VUS — functional validation would strengthen the case; (3) no BAM available for rigorous SV/CNV calling (GATK-SV, Manta); (4) mosaic somatic variants below ~20% VAF may be missed by the upstream short-read caller.
 The method scales naturally to cohorts by iterating the three configurations per proband and generalizes to any rare Mendelian phenotype with a defined HPO profile. Code and configuration files will be released publicly at the end of the hackathon.</t>
         </is>

</xml_diff>